<commit_message>
made changes to 9000+ combinations
</commit_message>
<xml_diff>
--- a/Estate_Path_Combinations_With_Roadmap.xlsx
+++ b/Estate_Path_Combinations_With_Roadmap.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aravi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aravi\Documents\AI_LLM\projects\exact-screenshot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3739C61A-D6FC-4F81-B6D0-1912A7692711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58135CB6-AE22-4F7B-83F7-398836003612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -926,6 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M193"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -984,7 +985,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1025,7 +1026,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1066,7 +1067,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1107,7 +1108,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1148,7 +1149,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1189,7 +1190,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1230,7 +1231,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1271,7 +1272,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1312,7 +1313,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1353,7 +1354,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1394,7 +1395,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1435,7 +1436,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1517,7 +1518,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1558,7 +1559,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1599,7 +1600,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1640,7 +1641,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1722,7 +1723,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -1763,7 +1764,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1804,7 +1805,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1845,7 +1846,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1886,7 +1887,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -1927,7 +1928,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -1968,7 +1969,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -2009,7 +2010,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -2050,7 +2051,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -2091,7 +2092,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -2132,7 +2133,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -2173,7 +2174,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -2214,7 +2215,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -2255,7 +2256,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -2296,7 +2297,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -2337,7 +2338,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -2378,7 +2379,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -2460,7 +2461,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -2501,7 +2502,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -2542,7 +2543,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -2583,7 +2584,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -2624,7 +2625,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -2665,7 +2666,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -2706,7 +2707,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -2747,7 +2748,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -2788,7 +2789,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -2829,7 +2830,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -2870,7 +2871,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -2911,7 +2912,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -2993,7 +2994,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -3034,7 +3035,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -3075,7 +3076,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -3116,7 +3117,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -3157,7 +3158,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -3198,7 +3199,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -3239,7 +3240,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -3280,7 +3281,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -3321,7 +3322,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -3362,7 +3363,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -3403,7 +3404,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -3485,7 +3486,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -3526,7 +3527,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -3567,7 +3568,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -3608,7 +3609,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -3649,7 +3650,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -3690,7 +3691,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -3731,7 +3732,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -3772,7 +3773,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -3813,7 +3814,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -3854,7 +3855,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -3895,7 +3896,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -3936,7 +3937,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -3977,7 +3978,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -4018,7 +4019,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -4059,7 +4060,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -4100,7 +4101,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -4141,7 +4142,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -4182,7 +4183,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -4223,7 +4224,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -4264,7 +4265,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -4305,7 +4306,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -4346,7 +4347,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -4387,7 +4388,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -4469,7 +4470,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -4510,7 +4511,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -4551,7 +4552,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -4592,7 +4593,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>13</v>
       </c>
@@ -4633,7 +4634,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>13</v>
       </c>
@@ -4674,7 +4675,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>13</v>
       </c>
@@ -4715,7 +4716,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>13</v>
       </c>
@@ -4756,7 +4757,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>13</v>
       </c>
@@ -4797,7 +4798,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>13</v>
       </c>
@@ -4838,7 +4839,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -4879,7 +4880,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -4920,7 +4921,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>26</v>
       </c>
@@ -4961,7 +4962,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>26</v>
       </c>
@@ -5002,7 +5003,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>26</v>
       </c>
@@ -5043,7 +5044,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>26</v>
       </c>
@@ -5084,7 +5085,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>26</v>
       </c>
@@ -5125,7 +5126,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>26</v>
       </c>
@@ -5166,7 +5167,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>26</v>
       </c>
@@ -5207,7 +5208,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>26</v>
       </c>
@@ -5248,7 +5249,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>26</v>
       </c>
@@ -5289,7 +5290,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>26</v>
       </c>
@@ -5330,7 +5331,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>26</v>
       </c>
@@ -5371,7 +5372,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>26</v>
       </c>
@@ -5412,7 +5413,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>26</v>
       </c>
@@ -5453,7 +5454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>26</v>
       </c>
@@ -5494,7 +5495,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>26</v>
       </c>
@@ -5535,7 +5536,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>26</v>
       </c>
@@ -5576,7 +5577,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>26</v>
       </c>
@@ -5617,7 +5618,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>26</v>
       </c>
@@ -5658,7 +5659,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>26</v>
       </c>
@@ -5699,7 +5700,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>26</v>
       </c>
@@ -5740,7 +5741,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>26</v>
       </c>
@@ -5781,7 +5782,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>26</v>
       </c>
@@ -5822,7 +5823,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>26</v>
       </c>
@@ -5863,7 +5864,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>26</v>
       </c>
@@ -5904,7 +5905,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>26</v>
       </c>
@@ -5945,7 +5946,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>26</v>
       </c>
@@ -5986,7 +5987,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>26</v>
       </c>
@@ -6027,7 +6028,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>26</v>
       </c>
@@ -6068,7 +6069,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>26</v>
       </c>
@@ -6109,7 +6110,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>26</v>
       </c>
@@ -6150,7 +6151,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>26</v>
       </c>
@@ -6191,7 +6192,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>26</v>
       </c>
@@ -6232,7 +6233,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>26</v>
       </c>
@@ -6273,7 +6274,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>26</v>
       </c>
@@ -6314,7 +6315,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>26</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>26</v>
       </c>
@@ -6396,7 +6397,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>26</v>
       </c>
@@ -6437,7 +6438,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>26</v>
       </c>
@@ -6478,7 +6479,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>26</v>
       </c>
@@ -6519,7 +6520,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>26</v>
       </c>
@@ -6560,7 +6561,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>26</v>
       </c>
@@ -6601,7 +6602,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>26</v>
       </c>
@@ -6642,7 +6643,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>26</v>
       </c>
@@ -6683,7 +6684,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>26</v>
       </c>
@@ -6724,7 +6725,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>26</v>
       </c>
@@ -6765,7 +6766,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>26</v>
       </c>
@@ -6806,7 +6807,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>26</v>
       </c>
@@ -6847,7 +6848,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>26</v>
       </c>
@@ -6929,7 +6930,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>26</v>
       </c>
@@ -6970,7 +6971,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>26</v>
       </c>
@@ -7011,7 +7012,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>26</v>
       </c>
@@ -7052,7 +7053,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>26</v>
       </c>
@@ -7093,7 +7094,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>26</v>
       </c>
@@ -7134,7 +7135,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>26</v>
       </c>
@@ -7175,7 +7176,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>26</v>
       </c>
@@ -7216,7 +7217,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>26</v>
       </c>
@@ -7257,7 +7258,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>26</v>
       </c>
@@ -7298,7 +7299,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -7339,7 +7340,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>26</v>
       </c>
@@ -7421,7 +7422,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>26</v>
       </c>
@@ -7462,7 +7463,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>26</v>
       </c>
@@ -7503,7 +7504,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>26</v>
       </c>
@@ -7544,7 +7545,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>26</v>
       </c>
@@ -7585,7 +7586,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>26</v>
       </c>
@@ -7626,7 +7627,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>26</v>
       </c>
@@ -7667,7 +7668,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>26</v>
       </c>
@@ -7708,7 +7709,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>26</v>
       </c>
@@ -7749,7 +7750,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>26</v>
       </c>
@@ -7790,7 +7791,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>26</v>
       </c>
@@ -7831,7 +7832,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>26</v>
       </c>
@@ -7872,7 +7873,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>26</v>
       </c>
@@ -7913,7 +7914,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>26</v>
       </c>
@@ -7954,7 +7955,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>26</v>
       </c>
@@ -7995,7 +7996,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>26</v>
       </c>
@@ -8036,7 +8037,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>26</v>
       </c>
@@ -8077,7 +8078,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>26</v>
       </c>
@@ -8118,7 +8119,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>26</v>
       </c>
@@ -8159,7 +8160,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>26</v>
       </c>
@@ -8200,7 +8201,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>26</v>
       </c>
@@ -8241,7 +8242,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>26</v>
       </c>
@@ -8282,7 +8283,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>26</v>
       </c>
@@ -8323,7 +8324,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>26</v>
       </c>
@@ -8364,7 +8365,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>26</v>
       </c>
@@ -8405,7 +8406,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>26</v>
       </c>
@@ -8446,7 +8447,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>26</v>
       </c>
@@ -8487,7 +8488,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>26</v>
       </c>
@@ -8528,7 +8529,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>26</v>
       </c>
@@ -8569,7 +8570,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>26</v>
       </c>
@@ -8610,7 +8611,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>26</v>
       </c>
@@ -8651,7 +8652,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>26</v>
       </c>
@@ -8692,7 +8693,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>26</v>
       </c>
@@ -8733,7 +8734,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>26</v>
       </c>
@@ -8774,7 +8775,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>26</v>
       </c>
@@ -8815,7 +8816,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>26</v>
       </c>
@@ -8857,7 +8858,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M193" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M193" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Ancillary Probate Required"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Harden roadmap track gating and align sidebar/legal path flows
</commit_message>
<xml_diff>
--- a/Estate_Path_Combinations_With_Roadmap.xlsx
+++ b/Estate_Path_Combinations_With_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aravi\Documents\AI_LLM\projects\exact-screenshot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58135CB6-AE22-4F7B-83F7-398836003612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EA8240-B930-4E62-AC8E-A6B75900B5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -926,7 +926,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:M193"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -985,7 +984,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1026,7 +1025,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1067,7 +1066,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1108,7 +1107,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1149,7 +1148,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1190,7 +1189,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1231,7 +1230,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1272,7 +1271,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1313,7 +1312,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1354,7 +1353,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1395,7 +1394,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1436,7 +1435,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1477,7 +1476,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1518,7 +1517,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1559,7 +1558,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1600,7 +1599,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1641,7 +1640,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1723,7 +1722,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -1764,7 +1763,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1805,7 +1804,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1846,7 +1845,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1887,7 +1886,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -1928,7 +1927,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -1969,7 +1968,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -2010,7 +2009,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -2051,7 +2050,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -2092,7 +2091,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -2133,7 +2132,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -2174,7 +2173,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -2215,7 +2214,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -2256,7 +2255,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -2297,7 +2296,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -2338,7 +2337,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -2379,7 +2378,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -2420,7 +2419,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -2461,7 +2460,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -2502,7 +2501,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -2543,7 +2542,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -2584,7 +2583,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -2625,7 +2624,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -2666,7 +2665,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -2707,7 +2706,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -2748,7 +2747,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -2789,7 +2788,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -2830,7 +2829,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -2871,7 +2870,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -2912,7 +2911,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -2994,7 +2993,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -3035,7 +3034,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -3076,7 +3075,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -3117,7 +3116,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -3158,7 +3157,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -3199,7 +3198,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -3240,7 +3239,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -3281,7 +3280,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -3322,7 +3321,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -3363,7 +3362,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -3404,7 +3403,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -3486,7 +3485,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -3527,7 +3526,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -3568,7 +3567,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -3609,7 +3608,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -3650,7 +3649,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -3691,7 +3690,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -3732,7 +3731,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -3773,7 +3772,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -3814,7 +3813,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -3855,7 +3854,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -3896,7 +3895,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -3937,7 +3936,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -3978,7 +3977,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -4019,7 +4018,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -4060,7 +4059,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -4101,7 +4100,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -4142,7 +4141,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -4183,7 +4182,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -4224,7 +4223,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -4265,7 +4264,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -4306,7 +4305,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -4347,7 +4346,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="84" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -4388,7 +4387,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -4429,7 +4428,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -4470,7 +4469,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="87" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -4511,7 +4510,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="88" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -4552,7 +4551,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="89" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -4593,7 +4592,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="90" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>13</v>
       </c>
@@ -4634,7 +4633,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="91" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>13</v>
       </c>
@@ -4675,7 +4674,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="92" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>13</v>
       </c>
@@ -4716,7 +4715,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>13</v>
       </c>
@@ -4757,7 +4756,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="94" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>13</v>
       </c>
@@ -4798,7 +4797,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="95" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>13</v>
       </c>
@@ -4839,7 +4838,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="96" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -4880,7 +4879,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -4921,7 +4920,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>26</v>
       </c>
@@ -4962,7 +4961,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>26</v>
       </c>
@@ -5003,7 +5002,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>26</v>
       </c>
@@ -5044,7 +5043,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>26</v>
       </c>
@@ -5085,7 +5084,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>26</v>
       </c>
@@ -5126,7 +5125,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>26</v>
       </c>
@@ -5167,7 +5166,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>26</v>
       </c>
@@ -5208,7 +5207,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>26</v>
       </c>
@@ -5249,7 +5248,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>26</v>
       </c>
@@ -5290,7 +5289,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>26</v>
       </c>
@@ -5331,7 +5330,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>26</v>
       </c>
@@ -5372,7 +5371,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>26</v>
       </c>
@@ -5413,7 +5412,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>26</v>
       </c>
@@ -5454,7 +5453,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>26</v>
       </c>
@@ -5495,7 +5494,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>26</v>
       </c>
@@ -5536,7 +5535,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>26</v>
       </c>
@@ -5577,7 +5576,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="114" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>26</v>
       </c>
@@ -5618,7 +5617,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>26</v>
       </c>
@@ -5659,7 +5658,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>26</v>
       </c>
@@ -5700,7 +5699,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>26</v>
       </c>
@@ -5741,7 +5740,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>26</v>
       </c>
@@ -5782,7 +5781,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>26</v>
       </c>
@@ -5823,7 +5822,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>26</v>
       </c>
@@ -5864,7 +5863,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>26</v>
       </c>
@@ -5905,7 +5904,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>26</v>
       </c>
@@ -5946,7 +5945,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="123" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>26</v>
       </c>
@@ -5987,7 +5986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>26</v>
       </c>
@@ -6028,7 +6027,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>26</v>
       </c>
@@ -6069,7 +6068,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>26</v>
       </c>
@@ -6110,7 +6109,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>26</v>
       </c>
@@ -6151,7 +6150,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>26</v>
       </c>
@@ -6192,7 +6191,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>26</v>
       </c>
@@ -6233,7 +6232,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>26</v>
       </c>
@@ -6274,7 +6273,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>26</v>
       </c>
@@ -6315,7 +6314,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>26</v>
       </c>
@@ -6356,7 +6355,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>26</v>
       </c>
@@ -6397,7 +6396,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>26</v>
       </c>
@@ -6438,7 +6437,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>26</v>
       </c>
@@ -6479,7 +6478,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>26</v>
       </c>
@@ -6520,7 +6519,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>26</v>
       </c>
@@ -6561,7 +6560,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>26</v>
       </c>
@@ -6602,7 +6601,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="139" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>26</v>
       </c>
@@ -6643,7 +6642,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="140" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>26</v>
       </c>
@@ -6684,7 +6683,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="141" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>26</v>
       </c>
@@ -6725,7 +6724,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="142" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>26</v>
       </c>
@@ -6766,7 +6765,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="143" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>26</v>
       </c>
@@ -6807,7 +6806,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="144" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>26</v>
       </c>
@@ -6848,7 +6847,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="145" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>26</v>
       </c>
@@ -6930,7 +6929,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="147" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>26</v>
       </c>
@@ -6971,7 +6970,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="148" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>26</v>
       </c>
@@ -7012,7 +7011,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="149" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>26</v>
       </c>
@@ -7053,7 +7052,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="150" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>26</v>
       </c>
@@ -7094,7 +7093,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="151" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>26</v>
       </c>
@@ -7135,7 +7134,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="152" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>26</v>
       </c>
@@ -7176,7 +7175,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="153" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>26</v>
       </c>
@@ -7217,7 +7216,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="154" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>26</v>
       </c>
@@ -7258,7 +7257,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="155" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>26</v>
       </c>
@@ -7299,7 +7298,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="156" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -7340,7 +7339,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="157" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>26</v>
       </c>
@@ -7422,7 +7421,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="159" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>26</v>
       </c>
@@ -7463,7 +7462,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="160" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>26</v>
       </c>
@@ -7504,7 +7503,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="161" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>26</v>
       </c>
@@ -7545,7 +7544,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="162" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>26</v>
       </c>
@@ -7586,7 +7585,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="163" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>26</v>
       </c>
@@ -7627,7 +7626,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="164" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>26</v>
       </c>
@@ -7668,7 +7667,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="165" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>26</v>
       </c>
@@ -7709,7 +7708,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="166" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>26</v>
       </c>
@@ -7750,7 +7749,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="167" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>26</v>
       </c>
@@ -7791,7 +7790,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="168" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>26</v>
       </c>
@@ -7832,7 +7831,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="169" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>26</v>
       </c>
@@ -7873,7 +7872,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="170" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>26</v>
       </c>
@@ -7914,7 +7913,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="171" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>26</v>
       </c>
@@ -7955,7 +7954,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="172" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>26</v>
       </c>
@@ -7996,7 +7995,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="173" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>26</v>
       </c>
@@ -8037,7 +8036,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="174" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>26</v>
       </c>
@@ -8078,7 +8077,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="175" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>26</v>
       </c>
@@ -8119,7 +8118,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="176" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>26</v>
       </c>
@@ -8160,7 +8159,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="177" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>26</v>
       </c>
@@ -8201,7 +8200,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="178" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>26</v>
       </c>
@@ -8242,7 +8241,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="179" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>26</v>
       </c>
@@ -8283,7 +8282,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="180" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>26</v>
       </c>
@@ -8324,7 +8323,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="181" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>26</v>
       </c>
@@ -8365,7 +8364,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="182" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>26</v>
       </c>
@@ -8406,7 +8405,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="183" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>26</v>
       </c>
@@ -8447,7 +8446,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="184" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>26</v>
       </c>
@@ -8488,7 +8487,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="185" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>26</v>
       </c>
@@ -8529,7 +8528,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="186" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>26</v>
       </c>
@@ -8570,7 +8569,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="187" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>26</v>
       </c>
@@ -8611,7 +8610,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="188" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>26</v>
       </c>
@@ -8652,7 +8651,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="189" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>26</v>
       </c>
@@ -8693,7 +8692,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="190" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>26</v>
       </c>
@@ -8734,7 +8733,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="191" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>26</v>
       </c>
@@ -8775,7 +8774,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="192" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>26</v>
       </c>
@@ -8816,7 +8815,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="193" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>26</v>
       </c>
@@ -8858,13 +8857,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M193" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="Ancillary Probate Required"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M193" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>